<commit_message>
feat: extend financial indicator rule management and template import/export
</commit_message>
<xml_diff>
--- a/config/key_ratio_rulebook.xlsx
+++ b/config/key_ratio_rulebook.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1705,6 +1705,428 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>roe_method_note</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>分解方法：采用Shapley分解（乘法体系），按三因子对ROE变动的边际贡献进行公平分摊。</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>???????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>roe_contrib_detail</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>三因子贡献：净利率{nm_contrib}个百分点（驱动占比{nm_share}），总资产周转率{at_contrib}个百分点（驱动占比{at_share}），权益乘数{em_contrib}个百分点（驱动占比{em_share}）。</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>??????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>roe_reconcile</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>分解校验：三因子贡献合计{contrib_sum}个百分点，对应ROE变动{roe_delta}个百分点。</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>?????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>trend_word_up</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>wording</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>上升</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>ROE/????????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>trend_word_down</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>wording</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>下降</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ROE/????????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>trend_word_stable</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>wording</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>基本稳定</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>ROE/????????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>roe_missing_years</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>杜邦分析所需年度不足，待补充。</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>ROE??-???</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>gm_missing_years</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>毛利率贡献分析所需年度不足，待补充。</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>?????-???</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>gm_missing_segments</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>未识别到营业收入分项，毛利率贡献待补充。</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>?????-???</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>gm_negative_impact_summary</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>各分项按绝对影响占比展示，不采用简单占比</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>??????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>gm_segment_header</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>???????{y1}-{y3}??</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>y1,y3</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>?????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>gm_segment_line</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>{name}???{ds}???????/??{dm}???????{di}???????{dt}??????????{net_share}???????{strength_share}?</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>name,ds,dm,di,dt,net_share,strength_share</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>gm_segment_summary</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>???????????{top_pos}???????{top_neg}?</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>top_pos,top_neg</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>?????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>gm_net_share_na</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>??????????0?</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>???????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>gm_top_fallback</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>???Top?????</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>